<commit_message>
Ajusta regras de local e exclusao por ajuste
</commit_message>
<xml_diff>
--- a/utils/insumos/regra_ajuste_final.xlsx
+++ b/utils/insumos/regra_ajuste_final.xlsx
@@ -407,7 +407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="4" min="1" max="1"/>
@@ -438,72 +438,77 @@
           <t>ORDEM</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ACAO</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>VALOR_ATUAL_ESPERADO</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>COMPARADOR_1</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>VALOR_1</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_2</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>COMPARADOR_2</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>VALOR_2</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_3</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>COMPARADOR_3</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>VALOR_3</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
@@ -518,56 +523,61 @@
       <c r="B2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>HOSPITAL SAO LUCAS</t>
         </is>
       </c>
-      <c r="E2" s="7" t="n"/>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>LOCAL</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>NOTRE DAME INTERMEDICA SAUDE SA; NOTRE DAME INTERMEDICA SAUDE S A; NOTRE DAME INTERMEDICA SAUDE S.A.; NOTRE DAME INTERMEDICA SAUDE S.A; NOTRE DAME INTERMEDICA SAUDE S; NOTRE DAME INTERMEDICA SAUDE</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="M2" s="7" t="n"/>
       <c r="N2" s="7" t="n"/>
       <c r="O2" s="7" t="n"/>
-      <c r="P2" s="7" t="inlineStr">
+      <c r="P2" s="7" t="n"/>
+      <c r="Q2" s="7" t="inlineStr">
         <is>
           <t>Ajusta Notre Dame SP para Hospital Sao Lucas</t>
         </is>
@@ -582,32 +592,37 @@
       <c r="B3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>HOSPITAL ILHA DO LEITE</t>
         </is>
@@ -622,32 +637,37 @@
       <c r="B4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>RN</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>HOSPITAL ANTONIO PRUDENTE NATAL</t>
         </is>
@@ -662,32 +682,37 @@
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>HOSPITAL CRUZEIRO DO SUL</t>
         </is>
@@ -702,32 +727,37 @@
       <c r="B6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>HOSPITAL E MATERNIDADE SALVALUS</t>
         </is>
@@ -742,34 +772,74 @@
       <c r="B7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>HOSPITAL SAO JOSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>excluir</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CLASSIFICACAO</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>AMBULANCIA</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Exclui classificacao ambulancia</t>
         </is>
       </c>
     </row>
@@ -916,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="5" min="1" max="1"/>
@@ -932,411 +1002,435 @@
       <c r="B1" s="8" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Ideia geral</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Cada linha ativa da aba regras_ajuste_final aplica um ajuste quando todos os filtros informados forem verdadeiros.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Colunas principais</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>STATUS_ATIVO</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>sim ativa a regra; vazio ou nao desativa.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>ORDEM</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Define a ordem de aplicacao. Regras menores rodam primeiro.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Coluna da base que recebera o ajuste, por exemplo LOCAL EDITADO ou UF.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Texto fixo a gravar ou COLUNA:NOME_DA_COLUNA para copiar valor linha a linha.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>VALOR_ATUAL_ESPERADO</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Opcional. Se preenchido, so altera quando a coluna ajustada ja tiver esse valor.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>sim permite alterar valor existente; nao altera apenas quando a coluna ajustada esta vazia.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1/2/3</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Colunas usadas como condicao para a regra.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>COMPARADOR_1/2/3</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Operacao do filtro: igual, diferente, em_lista, fora_lista, contem, nao_contem, vazio, nao_vazio.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>VALOR_1/2/3</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Valor usado pelo filtro. Em em_lista, separe valores com ponto e virgula.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Texto livre para identificar a regra nos resumos e auditoria.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Exemplo 1 - valor fixo</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Objetivo: quando LOCAL EDITADO for HOSPITAL ANA LIMA e UF estiver vazia, preencher UF com CE.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>CE</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>nao</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>COMPARADOR_1</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>VALOR_1</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>HOSPITAL ANA LIMA</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Exemplo 2 - copiar valor de outra coluna</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Objetivo: quando CLASSIFICACAO = ODONTOLOGIA, TIPO = 5 e LOCAL EDITADO estiver vazio, preencher LOCAL EDITADO com PROFISSIONAL.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>COLUNA:PROFISSIONAL</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>nao</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>CLASSIFICACAO</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>COMPARADOR_1</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>VALOR_1</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>ODONTOLOGIA</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_2</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>TIPO</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>COMPARADOR_2</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>VALOR_2</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_3</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>COMPARADOR_3</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>vazio</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
+      <c r="A40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Observacao sobre COLUNA:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>COLUNA:PROFISSIONAL copia o valor correspondente da coluna PROFISSIONAL em cada linha atingida.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>Valores fixos continuam funcionando normalmente, por exemplo VALOR_NOVO = SP ou VALOR_NOVO = ODONTOLOGIA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ACAO</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Use 'ajustar' para alterar valores ou 'excluir' para remover as linhas que baterem nos filtros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Exemplo - excluir linhas</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ACAO = excluir, COLUNA_FILTRO_1 = CLASSIFICACAO, COMPARADOR_1 = igual, VALOR_1 = AMBULANCIA.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona consulta Oracle de quantidades
</commit_message>
<xml_diff>
--- a/utils/insumos/regra_ajuste_final.xlsx
+++ b/utils/insumos/regra_ajuste_final.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-180" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regras_ajuste_final" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,14 +14,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'regras_ajuste_final'!$A$1:$P$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'comparadores'!$A$1:$B$9</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -31,24 +30,8 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="0"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <name val="Cambria"/>
       <charset val="1"/>
-      <family val="0"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
@@ -60,6 +43,11 @@
       <color theme="3"/>
       <sz val="18"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <name val="Arial Unicode MS"/>
+      <color theme="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -85,84 +73,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="6"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
-    <cellStyle name="Currency" xfId="3" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Percent" xfId="5" builtinId="5"/>
-    <cellStyle name="Title" xfId="6" builtinId="15" hidden="0"/>
+    <cellStyle name="Título" xfId="1" builtinId="15"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F4E78"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -221,47 +153,55 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E78"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -269,12 +209,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -303,7 +243,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -324,7 +264,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -375,7 +315,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -393,47 +333,49 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:Q10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="15" customWidth="1" style="4" min="1" max="1"/>
-    <col width="10" customWidth="1" style="4" min="2" max="2"/>
-    <col width="20" customWidth="1" style="4" min="3" max="3"/>
-    <col width="28" customWidth="1" style="4" min="4" max="5"/>
-    <col width="30.32" customWidth="1" style="4" min="6" max="6"/>
-    <col width="20" customWidth="1" style="4" min="7" max="7"/>
-    <col width="24.49" customWidth="1" style="4" min="8" max="8"/>
-    <col width="65" customWidth="1" style="4" min="9" max="9"/>
-    <col width="20" customWidth="1" style="4" min="10" max="10"/>
-    <col width="16" customWidth="1" style="4" min="11" max="11"/>
-    <col width="18" customWidth="1" style="4" min="12" max="12"/>
-    <col width="20" customWidth="1" style="4" min="13" max="13"/>
-    <col width="16" customWidth="1" style="4" min="14" max="14"/>
-    <col width="28" customWidth="1" style="4" min="15" max="15"/>
-    <col width="50" customWidth="1" style="4" min="16" max="16"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="5"/>
+    <col width="30.28515625" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="24.42578125" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="38.85546875" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="50" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="5">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>STATUS_ATIVO</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ORDEM</t>
         </is>
@@ -443,84 +385,84 @@
           <t>ACAO</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>VALOR_ATUAL_ESPERADO</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR_1</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>VALOR_1</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_2</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR_2</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>VALOR_2</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_3</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR_3</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>VALOR_3</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18.65" customHeight="1" s="5">
-      <c r="A2" s="7" t="inlineStr">
+    <row r="2" ht="18.6" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -528,68 +470,68 @@
           <t>ajustar</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>HOSPITAL SAO LUCAS</t>
         </is>
       </c>
-      <c r="F2" s="7" t="n"/>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>LOCAL</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>NOTRE DAME INTERMEDICA SAUDE SA; NOTRE DAME INTERMEDICA SAUDE S A; NOTRE DAME INTERMEDICA SAUDE S.A.; NOTRE DAME INTERMEDICA SAUDE S.A; NOTRE DAME INTERMEDICA SAUDE S; NOTRE DAME INTERMEDICA SAUDE</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="N2" s="7" t="n"/>
-      <c r="O2" s="7" t="n"/>
-      <c r="P2" s="7" t="n"/>
-      <c r="Q2" s="7" t="inlineStr">
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Ajusta Notre Dame SP para Hospital Sao Lucas</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="5">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -597,44 +539,44 @@
           <t>ajustar</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>HOSPITAL ILHA DO LEITE</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="5">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -642,44 +584,44 @@
           <t>ajustar</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>RN</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>HOSPITAL ANTONIO PRUDENTE NATAL</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -687,122 +629,122 @@
           <t>ajustar</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>HOSPITAL CRUZEIRO DO SUL</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="5">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>4</v>
+      <c r="B6" t="n">
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>ajustar</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>HOSPITAL E MATERNIDADE SALVALUS</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="5">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>4</v>
+      <c r="B7" t="n">
+        <v>6</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>ajustar</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>HOSPITAL SAO JOSE</t>
         </is>
@@ -815,7 +757,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -840,133 +782,280 @@
       <c r="Q8" t="inlineStr">
         <is>
           <t>Exclui classificacao ambulancia</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CONTRATACAO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>rede credenciada</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>LOCAL EDITADO</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Igual</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>HAPVIDA ASSISTENCIA MEDICA S.A</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>CLASSIFICACAO</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>ODONTOLOGIA</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>realocando classificações odonto para rede credenciada</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ajustar</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LOCAL EDITADO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>COLUNA:PROFISSIONAL</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>n?o</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>CLASSIFICACAO</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ODONTOLOGIA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>LOCAL EDITADO</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>vazio</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>LOCAL</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>igual</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Para odontologia sem local, usa profissional como local editado</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P2"/>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;1 &amp;KFF0000 INTERNO#_x000d_</oddHeader>
+    <oddFooter>&amp;C&amp;"Aptos"&amp;10 &amp;KFF0000_x000d_# INTERNO</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="18" customWidth="1" style="4" min="1" max="1"/>
-    <col width="80" customWidth="1" style="4" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="5">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>COMPARADOR</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="5">
-      <c r="A2" s="7" t="inlineStr">
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Valor da coluna deve ser igual ao valor informado.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="5">
-      <c r="A3" s="7" t="inlineStr">
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>diferente</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Valor da coluna deve ser diferente do valor informado.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="5">
-      <c r="A4" s="7" t="inlineStr">
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>em_lista</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Valor da coluna deve estar em lista separada por ponto e virgula.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="5">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>fora_lista</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Valor da coluna nao deve estar em lista separada por ponto e virgula.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="5">
-      <c r="A6" s="7" t="inlineStr">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>contem</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Texto da coluna deve conter o valor informado.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="5">
-      <c r="A7" s="7" t="inlineStr">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>nao_contem</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Texto da coluna nao deve conter o valor informado.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="5">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>vazio</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Coluna deve estar vazia.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="5">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>nao_vazio</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Coluna nao deve estar vazia.</t>
         </is>
@@ -974,9 +1063,16 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:B9"/>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;1 &amp;KFF0000 INTERNO#_x000d_</oddHeader>
+    <oddFooter>&amp;C&amp;"Aptos"&amp;10 &amp;KFF0000_x000d_# INTERNO</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -989,422 +1085,407 @@
   <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="5" min="1" max="1"/>
-    <col width="115" customWidth="1" style="5" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>TUTORIAL - REGRAS DE AJUSTE FINAL</t>
         </is>
       </c>
-      <c r="B1" s="8" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B1" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Ideia geral</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Cada linha ativa da aba regras_ajuste_final aplica um ajuste quando todos os filtros informados forem verdadeiros.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr"/>
-    </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Colunas principais</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>STATUS_ATIVO</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>sim ativa a regra; vazio ou nao desativa.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>ORDEM</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Define a ordem de aplicacao. Regras menores rodam primeiro.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Coluna da base que recebera o ajuste, por exemplo LOCAL EDITADO ou UF.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Texto fixo a gravar ou COLUNA:NOME_DA_COLUNA para copiar valor linha a linha.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>VALOR_ATUAL_ESPERADO</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Opcional. Se preenchido, so altera quando a coluna ajustada ja tiver esse valor.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>sim permite alterar valor existente; nao altera apenas quando a coluna ajustada esta vazia.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1/2/3</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Colunas usadas como condicao para a regra.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>COMPARADOR_1/2/3</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Operacao do filtro: igual, diferente, em_lista, fora_lista, contem, nao_contem, vazio, nao_vazio.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>VALOR_1/2/3</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Valor usado pelo filtro. Em em_lista, separe valores com ponto e virgula.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Texto livre para identificar a regra nos resumos e auditoria.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Exemplo 1 - valor fixo</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Objetivo: quando LOCAL EDITADO for HOSPITAL ANA LIMA e UF estiver vazia, preencher UF com CE.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>CE</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>nao</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>COMPARADOR_1</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>VALOR_1</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>HOSPITAL ANA LIMA</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Exemplo 2 - copiar valor de outra coluna</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Objetivo: quando CLASSIFICACAO = ODONTOLOGIA, TIPO = 5 e LOCAL EDITADO estiver vazio, preencher LOCAL EDITADO com PROFISSIONAL.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>COLUNA_AJUSTAR</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>VALOR_NOVO</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>COLUNA:PROFISSIONAL</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>PERMITIR_SOBRESCRITA</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>nao</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_1</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>CLASSIFICACAO</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>COMPARADOR_1</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>VALOR_1</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>ODONTOLOGIA</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_2</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>TIPO</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>COMPARADOR_2</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>igual</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>VALOR_2</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>COLUNA_FILTRO_3</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>LOCAL EDITADO</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>COMPARADOR_3</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>vazio</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr"/>
-    </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Observacao sobre COLUNA:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>COLUNA:PROFISSIONAL copia o valor correspondente da coluna PROFISSIONAL em cada linha atingida.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Valores fixos continuam funcionando normalmente, por exemplo VALOR_NOVO = SP ou VALOR_NOVO = ODONTOLOGIA.</t>
         </is>
@@ -1436,5 +1517,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;1 &amp;KFF0000 INTERNO#_x000d_</oddHeader>
+    <oddFooter>&amp;C&amp;"Aptos"&amp;10 &amp;KFF0000_x000d_# INTERNO</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>